<commit_message>
chore: update report outputs after tool verification run
</commit_message>
<xml_diff>
--- a/manual-testcases/News_CSS_Test_Cases_Results.xlsx
+++ b/manual-testcases/News_CSS_Test_Cases_Results.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="247">
   <si>
     <t>TC ID</t>
   </si>
@@ -83,16 +83,7 @@
     <t>Left and right gutters are equal on both sites. Values of max-width, margin, padding-left, padding-right match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>margin-top: 7.5px; margin-bottom: 7.5px; padding-left: 7.5px; padding-right: 7.5px</t>
-  </si>
-  <si>
-    <t>margin-top: 0px; margin-bottom: 0px; padding-left: 120px; padding-right: 120px</t>
-  </si>
-  <si>
     <t>Fail</t>
-  </si>
-  <si>
-    <t>margin-top (-7.50px), margin-bottom (-7.50px), padding-left (+112.50px), padding-right (+112.50px)</t>
   </si>
   <si>
     <t>TC02</t>
@@ -115,15 +106,6 @@
     <t>Top and bottom spacing is the same on both sites. Values of margin-top, margin-bottom, padding-top, padding-bottom match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>margin-top: 7.5px; margin-bottom: 7.5px; padding-top: 15px; padding-bottom: 15px</t>
-  </si>
-  <si>
-    <t>margin-top: 0px; margin-bottom: 0px; padding-top: 0px; padding-bottom: 0px</t>
-  </si>
-  <si>
-    <t>margin-top (-7.50px), margin-bottom (-7.50px), padding-top (-15.00px), padding-bottom (-15.00px)</t>
-  </si>
-  <si>
     <t>TC03</t>
   </si>
   <si>
@@ -150,15 +132,6 @@
     <t>Heading text style is identical on both sites. Values of font-size, font-weight, color match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>color: rgb(0, 50, 122)</t>
-  </si>
-  <si>
-    <t>color: rgb(0, 36, 143)</t>
-  </si>
-  <si>
-    <t>color (changed)</t>
-  </si>
-  <si>
     <t>TC04</t>
   </si>
   <si>
@@ -182,15 +155,6 @@
     <t>Heading is at the left and More button at the right, vertically aligned. Values of display, justify-content, align-items match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>display: block; justify-content: normal; align-items: normal</t>
-  </si>
-  <si>
-    <t>Pass</t>
-  </si>
-  <si>
-    <t>All checked properties match within tolerance.</t>
-  </si>
-  <si>
     <t>TC05</t>
   </si>
   <si>
@@ -214,15 +178,6 @@
     <t>Border width, style, color and radius are identical. Values of border, border-radius match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>border-top-width: 1px; border-right-width: 1px; border-bottom-width: 1px; border-left-width: 1px; border-top-left-radius: 5px; border-top-right-radius: 5px; border-bottom-right-radius: 5px; border-bottom-left-radius: 5px</t>
-  </si>
-  <si>
-    <t>border-top-width: 2px; border-right-width: 2px; border-bottom-width: 2px; border-left-width: 2px; border-top-left-radius: 8px; border-top-right-radius: 8px; border-bottom-right-radius: 8px; border-bottom-left-radius: 8px</t>
-  </si>
-  <si>
-    <t>border-top-width (+1.00px), border-right-width (+1.00px), border-bottom-width (+1.00px), border-left-width (+1.00px), border-top-left-radius (+3.00px), border-top-right-radius (+3.00px), border-bottom-right-radius (+3.00px), border-bottom-left-radius (+3.00px)</t>
-  </si>
-  <si>
     <t>TC06</t>
   </si>
   <si>
@@ -243,15 +198,6 @@
     <t>Button padding and text style are identical. Values of padding, font-size, font-weight, color match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>padding-top: 7.5px; padding-right: 7.5px; padding-bottom: 7.5px; padding-left: 7.5px; font-weight: 600; color: rgb(225, 10, 21)</t>
-  </si>
-  <si>
-    <t>padding-top: 4px; padding-right: 8px; padding-bottom: 4px; padding-left: 8px; font-weight: 700; color: rgb(221, 8, 22)</t>
-  </si>
-  <si>
-    <t>padding-top (-3.50px), padding-right (+0.50px), padding-bottom (-3.50px), padding-left (+0.50px), font-weight (changed), color (changed)</t>
-  </si>
-  <si>
     <t>TC07</t>
   </si>
   <si>
@@ -278,15 +224,6 @@
     <t>Both cards have the same width on each site and match across sites. Values of display, grid-template-columns, width match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>width: 547.5px</t>
-  </si>
-  <si>
-    <t>width: 592px</t>
-  </si>
-  <si>
-    <t>width (+44.50px)</t>
-  </si>
-  <si>
     <t>TC08</t>
   </si>
   <si>
@@ -307,15 +244,6 @@
     <t>Both cards have the same height on each site and match across sites. Values of height, aspect-ratio match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>height: 307.969px; aspect-ratio: auto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">height: 253.703px; aspect-ratio: </t>
-  </si>
-  <si>
-    <t>height (-54.27px), aspect-ratio (changed)</t>
-  </si>
-  <si>
     <t>TC09</t>
   </si>
   <si>
@@ -339,15 +267,6 @@
     <t>Gap between the two cards is identical. Values of gap, column-gap match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>gap: normal; column-gap: normal</t>
-  </si>
-  <si>
-    <t>gap: 16px; column-gap: 16px</t>
-  </si>
-  <si>
-    <t>gap (changed), column-gap (changed)</t>
-  </si>
-  <si>
     <t>TC10</t>
   </si>
   <si>
@@ -371,15 +290,6 @@
     <t>Image uses object-fit: cover and fills the card. Values of object-fit, width, height match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>object-fit: fill; width: 547.5px; height: 307.969px</t>
-  </si>
-  <si>
-    <t>object-fit: contain; width: 592px; height: 253.703px</t>
-  </si>
-  <si>
-    <t>object-fit (changed), width (+44.50px), height (-54.27px)</t>
-  </si>
-  <si>
     <t>TC11</t>
   </si>
   <si>
@@ -403,9 +313,6 @@
     <t>Title is positioned at the bottom-left over the image. Values of position, bottom, left, padding match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>position: static; bottom: auto; left: auto; padding-top: 0px</t>
-  </si>
-  <si>
     <t>TC12</t>
   </si>
   <si>
@@ -429,9 +336,6 @@
     <t>Title is white and a dark gradient or shadow sits behind it. Values of color, background-image, text-shadow match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>color: rgb(255, 255, 255); background-image: none; text-shadow: none</t>
-  </si>
-  <si>
     <t>TC13</t>
   </si>
   <si>
@@ -452,15 +356,6 @@
     <t>Title typography is identical on both sites. Values of font-size, font-weight, line-height match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>font-size: 20px; font-weight: 600; line-height: normal</t>
-  </si>
-  <si>
-    <t>font-size: 16px; font-weight: 700; line-height: 26px</t>
-  </si>
-  <si>
-    <t>font-size (-4.00px), font-weight (changed), line-height (changed)</t>
-  </si>
-  <si>
     <t>TC14</t>
   </si>
   <si>
@@ -481,9 +376,6 @@
     <t>Title is layered above the image. Values of z-index, position match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>z-index: auto; position: static</t>
-  </si>
-  <si>
     <t>TC15</t>
   </si>
   <si>
@@ -504,15 +396,6 @@
     <t>Long title stays inside the card, no overflow outside. Values of overflow, -webkit-line-clamp, word-break match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>-webkit-line-clamp: 3</t>
-  </si>
-  <si>
-    <t>-webkit-line-clamp: 2</t>
-  </si>
-  <si>
-    <t>-webkit-line-clamp (changed)</t>
-  </si>
-  <si>
     <t>TC16</t>
   </si>
   <si>
@@ -539,15 +422,6 @@
     <t>Four cards have equal width and sit in one row. Values of grid-template-columns, flex-basis, width match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>width: 266.25px</t>
-  </si>
-  <si>
-    <t>width: 288px</t>
-  </si>
-  <si>
-    <t>width (+21.75px)</t>
-  </si>
-  <si>
     <t>TC17</t>
   </si>
   <si>
@@ -591,15 +465,6 @@
     <t>All four images have the same height and no stretching. Values of height, aspect-ratio, object-fit match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>height: 149.766px; aspect-ratio: auto 400 / 225; object-fit: fill</t>
-  </si>
-  <si>
-    <t>height: 123.422px; aspect-ratio: auto; object-fit: contain</t>
-  </si>
-  <si>
-    <t>height (-26.34px), aspect-ratio (changed), object-fit (changed)</t>
-  </si>
-  <si>
     <t>TC19</t>
   </si>
   <si>
@@ -623,9 +488,6 @@
     <t>Title sits below the image with identical spacing. Values of margin-top, padding match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>margin-top: 0px; padding-top: 0px; padding-right: 0px; padding-bottom: 0px</t>
-  </si>
-  <si>
     <t>TC20</t>
   </si>
   <si>
@@ -646,15 +508,6 @@
     <t>Title typography is identical on both sites. Values of font-size, font-weight, color, line-height match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>font-size: 14px; font-weight: 600; color: rgb(0, 2, 13); line-height: normal</t>
-  </si>
-  <si>
-    <t>font-size: 18px; font-weight: 700; color: rgb(26, 26, 26); line-height: 24px</t>
-  </si>
-  <si>
-    <t>font-size (+4.00px), font-weight (changed), color (changed), line-height (changed)</t>
-  </si>
-  <si>
     <t>TC21</t>
   </si>
   <si>
@@ -675,9 +528,6 @@
     <t>Long title wraps or clamps without overlapping other content. Values of -webkit-line-clamp, overflow, text-overflow match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t xml:space="preserve">-webkit-line-clamp: </t>
-  </si>
-  <si>
     <t>TC22</t>
   </si>
   <si>
@@ -701,15 +551,6 @@
     <t>Vertical gap between the two rows is identical. Values of row-gap, margin-top match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>row-gap: normal; margin-top: 7.5px</t>
-  </si>
-  <si>
-    <t>row-gap: 16px; margin-top: 0px</t>
-  </si>
-  <si>
-    <t>row-gap (changed), margin-top (-7.50px)</t>
-  </si>
-  <si>
     <t>TC23</t>
   </si>
   <si>
@@ -736,15 +577,6 @@
     <t>Label size and color are identical. Values of font-size, color, opacity match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>font-size: 11px; color: rgba(255, 255, 255, 0.5)</t>
-  </si>
-  <si>
-    <t>font-size: 12px; color: rgb(175, 184, 197)</t>
-  </si>
-  <si>
-    <t>font-size (+1.00px), color (changed)</t>
-  </si>
-  <si>
     <t>TC24</t>
   </si>
   <si>
@@ -765,15 +597,6 @@
     <t>Label sits in the same position relative to the title. Values of margin, display, position match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>display: inline; position: static</t>
-  </si>
-  <si>
-    <t>display: flex; position: relative</t>
-  </si>
-  <si>
-    <t>display (changed), position (changed)</t>
-  </si>
-  <si>
     <t>TC25</t>
   </si>
   <si>
@@ -800,15 +623,6 @@
     <t>Button is fixed at the bottom-right corner. Values of position, right, bottom match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>position: relative; right: 0px; bottom: 0px</t>
-  </si>
-  <si>
-    <t>position: fixed; right: 24px; bottom: 24px</t>
-  </si>
-  <si>
-    <t>position (changed), right (+24.00px), bottom (+24.00px)</t>
-  </si>
-  <si>
     <t>TC26</t>
   </si>
   <si>
@@ -829,15 +643,6 @@
     <t>Button size and corner radius are identical. Values of width, height, border-radius match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>width: 40px; height: 40px; border-top-left-radius: 3px; border-top-right-radius: 3px; border-bottom-right-radius: 3px; border-bottom-left-radius: 3px</t>
-  </si>
-  <si>
-    <t>width: 44px; height: 44px; border-top-left-radius: 9999px; border-top-right-radius: 9999px; border-bottom-right-radius: 9999px; border-bottom-left-radius: 9999px</t>
-  </si>
-  <si>
-    <t>width (+4.00px), height (+4.00px), border-top-left-radius (+9996.00px), border-top-right-radius (+9996.00px), border-bottom-right-radius (+9996.00px), border-bottom-left-radius (+9996.00px)</t>
-  </si>
-  <si>
     <t>TC27</t>
   </si>
   <si>
@@ -858,15 +663,6 @@
     <t>Background and icon colors are identical. Values of background-color, color match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>background-color: rgb(245, 165, 0); color: rgb(0, 0, 0)</t>
-  </si>
-  <si>
-    <t>background-color: rgb(17, 17, 17); color: rgb(255, 255, 255)</t>
-  </si>
-  <si>
-    <t>background-color (changed), color (changed)</t>
-  </si>
-  <si>
     <t>TC28</t>
   </si>
   <si>
@@ -885,15 +681,6 @@
   </si>
   <si>
     <t>Button is layered above the page content. Values of z-index match on both sites (numeric tolerance +/-1px).</t>
-  </si>
-  <si>
-    <t>z-index: auto</t>
-  </si>
-  <si>
-    <t>z-index: 40</t>
-  </si>
-  <si>
-    <t>z-index (changed)</t>
   </si>
   <si>
     <t>TC29</t>
@@ -924,9 +711,6 @@
     <t>Hover effect (zoom or shadow) is identical on both sites. Values of transform, box-shadow, transition match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>transform: none; box-shadow: none; transition: all</t>
-  </si>
-  <si>
     <t>TC30</t>
   </si>
   <si>
@@ -952,9 +736,6 @@
     <t>Title color or underline on hover is identical. Values of color, text-decoration match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>color: rgb(255, 255, 255); text-decoration: none</t>
-  </si>
-  <si>
     <t>TC31</t>
   </si>
   <si>
@@ -977,12 +758,6 @@
     <t>Button hover state is identical. Values of background-color, color, cursor match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>background-color: rgba(0, 0, 0, 0); color: rgb(225, 10, 21)</t>
-  </si>
-  <si>
-    <t>background-color: rgb(242, 242, 242); color: rgb(221, 8, 22)</t>
-  </si>
-  <si>
     <t>TC32</t>
   </si>
   <si>
@@ -1004,9 +779,6 @@
   </si>
   <si>
     <t>Cursor is pointer on all clickable items. Values of cursor match on both sites (numeric tolerance +/-1px).</t>
-  </si>
-  <si>
-    <t>cursor: pointer</t>
   </si>
   <si>
     <t>TC33</t>
@@ -1030,15 +802,6 @@
     <t>Small cards show 2 per row at 768px. Values of grid-template-columns, flex-basis, width match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>grid-template-columns: none; width: 705px</t>
-  </si>
-  <si>
-    <t>grid-template-columns: 0px 0px 0px 0px 0px 0px 0px 0px 0px 191.328px 191.328px 191.328px; width: 750px</t>
-  </si>
-  <si>
-    <t>grid-template-columns (changed), width (+45.00px)</t>
-  </si>
-  <si>
     <t>TC34</t>
   </si>
   <si>
@@ -1063,15 +826,6 @@
     <t>All cards stack in 1 column at 375px. Values of grid-template-columns, flex-direction match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>grid-template-columns: none</t>
-  </si>
-  <si>
-    <t>grid-template-columns: 0px 0px 0px 0px 0px 0px 29.5px 29.5px 29.5px 26.1562px 26.1562px 26.1562px</t>
-  </si>
-  <si>
-    <t>grid-template-columns (changed)</t>
-  </si>
-  <si>
     <t>TC35</t>
   </si>
   <si>
@@ -1096,9 +850,6 @@
     <t>No horizontal scrollbar at 1440, 768 and 375px.</t>
   </si>
   <si>
-    <t>overflow-x: visible; scrollWidth: 1440px</t>
-  </si>
-  <si>
     <t>TC36</t>
   </si>
   <si>
@@ -1123,9 +874,6 @@
     <t>Font sizes at 375px are equal to or smaller than at 1440px and match across sites. Values of font-size match on both sites (numeric tolerance +/-1px).</t>
   </si>
   <si>
-    <t>font-size: 20px</t>
-  </si>
-  <si>
     <t>Item</t>
   </si>
   <si>
@@ -1190,6 +938,9 @@
   </si>
   <si>
     <t>Count</t>
+  </si>
+  <si>
+    <t>Pass</t>
   </si>
   <si>
     <t>Blocked</t>
@@ -1569,1278 +1320,1062 @@
         <v>18</v>
       </c>
       <c r="H2" s="2"/>
-      <c r="I2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>20</v>
-      </c>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
       <c r="K2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>22</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L2" s="2"/>
     </row>
     <row r="3" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>15</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="H3" s="2"/>
-      <c r="I3" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>29</v>
-      </c>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
       <c r="K3" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>30</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L3" s="2"/>
     </row>
     <row r="4" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>37</v>
-      </c>
       <c r="H4" s="2"/>
-      <c r="I4" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>39</v>
-      </c>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
       <c r="K4" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>40</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L4" s="2"/>
     </row>
     <row r="5" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="H5" s="2"/>
-      <c r="I5" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>47</v>
-      </c>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
       <c r="K5" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>49</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L5" s="2"/>
     </row>
     <row r="6" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="H6" s="2"/>
-      <c r="I6" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>57</v>
-      </c>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
       <c r="K6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>58</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L6" s="2"/>
     </row>
     <row r="7" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="H7" s="2"/>
-      <c r="I7" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>65</v>
-      </c>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
       <c r="K7" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>66</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L7" s="2"/>
     </row>
     <row r="8" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>69</v>
+        <v>51</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="H8" s="2"/>
-      <c r="I8" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>75</v>
-      </c>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
       <c r="K8" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>76</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L8" s="2"/>
     </row>
     <row r="9" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>79</v>
+        <v>58</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>80</v>
+        <v>59</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="H9" s="2"/>
-      <c r="I9" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>83</v>
-      </c>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
       <c r="K9" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L9" s="2" t="s">
-        <v>84</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L9" s="2"/>
     </row>
     <row r="10" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>85</v>
+        <v>61</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>86</v>
+        <v>62</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>87</v>
+        <v>63</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>89</v>
+        <v>65</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>90</v>
+        <v>66</v>
       </c>
       <c r="H10" s="2"/>
-      <c r="I10" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>92</v>
-      </c>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
       <c r="K10" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L10" s="2" t="s">
-        <v>93</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L10" s="2"/>
     </row>
     <row r="11" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>94</v>
+        <v>67</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>95</v>
-      </c>
       <c r="D11" s="2" t="s">
-        <v>96</v>
+        <v>69</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>97</v>
+        <v>70</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>98</v>
+        <v>71</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>99</v>
+        <v>72</v>
       </c>
       <c r="H11" s="2"/>
-      <c r="I11" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>101</v>
-      </c>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
       <c r="K11" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L11" s="2" t="s">
-        <v>102</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L11" s="2"/>
     </row>
     <row r="12" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>103</v>
+        <v>73</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>104</v>
+        <v>74</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>105</v>
+        <v>75</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>106</v>
+        <v>76</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>107</v>
+        <v>77</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>108</v>
+        <v>78</v>
       </c>
       <c r="H12" s="2"/>
-      <c r="I12" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>109</v>
-      </c>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
       <c r="K12" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="L12" s="2" t="s">
-        <v>49</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L12" s="2"/>
     </row>
     <row r="13" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>111</v>
+        <v>80</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>112</v>
+        <v>81</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>113</v>
+        <v>82</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>114</v>
+        <v>83</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>115</v>
+        <v>84</v>
       </c>
       <c r="H13" s="2"/>
-      <c r="I13" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>116</v>
-      </c>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
       <c r="K13" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="L13" s="2" t="s">
-        <v>49</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L13" s="2"/>
     </row>
     <row r="14" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>117</v>
+        <v>85</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>118</v>
+        <v>86</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>105</v>
+        <v>75</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>119</v>
+        <v>87</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>120</v>
+        <v>88</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>121</v>
+        <v>89</v>
       </c>
       <c r="H14" s="2"/>
-      <c r="I14" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>123</v>
-      </c>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
       <c r="K14" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L14" s="2" t="s">
-        <v>124</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L14" s="2"/>
     </row>
     <row r="15" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>125</v>
+        <v>90</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>126</v>
+        <v>91</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>105</v>
+        <v>75</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>127</v>
+        <v>92</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>128</v>
+        <v>93</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>129</v>
+        <v>94</v>
       </c>
       <c r="H15" s="2"/>
-      <c r="I15" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>130</v>
-      </c>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
       <c r="K15" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="L15" s="2" t="s">
-        <v>49</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L15" s="2"/>
     </row>
     <row r="16" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>131</v>
+        <v>95</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>132</v>
+        <v>96</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>105</v>
+        <v>75</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>133</v>
+        <v>97</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>134</v>
+        <v>98</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>135</v>
+        <v>99</v>
       </c>
       <c r="H16" s="2"/>
-      <c r="I16" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>137</v>
-      </c>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
       <c r="K16" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L16" s="2" t="s">
-        <v>138</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L16" s="2"/>
     </row>
     <row r="17" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>140</v>
+        <v>101</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>141</v>
+        <v>102</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>142</v>
+        <v>103</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>143</v>
+        <v>104</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>144</v>
+        <v>105</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>145</v>
+        <v>106</v>
       </c>
       <c r="H17" s="2"/>
-      <c r="I17" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>147</v>
-      </c>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
       <c r="K17" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L17" s="2" t="s">
-        <v>148</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L17" s="2"/>
     </row>
     <row r="18" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>149</v>
+        <v>107</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>140</v>
+        <v>101</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>150</v>
+        <v>108</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>151</v>
+        <v>109</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>152</v>
+        <v>110</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>153</v>
+        <v>111</v>
       </c>
       <c r="H18" s="2"/>
-      <c r="I18" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>92</v>
-      </c>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
       <c r="K18" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L18" s="2" t="s">
-        <v>93</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L18" s="2"/>
     </row>
     <row r="19" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>154</v>
+        <v>112</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>140</v>
+        <v>101</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>155</v>
+        <v>113</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>156</v>
+        <v>114</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>157</v>
+        <v>115</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>158</v>
+        <v>116</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>159</v>
+        <v>117</v>
       </c>
       <c r="H19" s="2"/>
-      <c r="I19" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>161</v>
-      </c>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
       <c r="K19" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L19" s="2" t="s">
-        <v>162</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L19" s="2"/>
     </row>
     <row r="20" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>163</v>
+        <v>118</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>140</v>
+        <v>101</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>164</v>
+        <v>119</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>165</v>
+        <v>120</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>166</v>
+        <v>121</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>167</v>
+        <v>122</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>168</v>
+        <v>123</v>
       </c>
       <c r="H20" s="2"/>
-      <c r="I20" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="J20" s="2" t="s">
-        <v>169</v>
-      </c>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
       <c r="K20" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="L20" s="2" t="s">
-        <v>49</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L20" s="2"/>
     </row>
     <row r="21" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>170</v>
+        <v>124</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>140</v>
+        <v>101</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>171</v>
+        <v>125</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>165</v>
+        <v>120</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>172</v>
+        <v>126</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>173</v>
+        <v>127</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>174</v>
+        <v>128</v>
       </c>
       <c r="H21" s="2"/>
-      <c r="I21" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="J21" s="2" t="s">
-        <v>176</v>
-      </c>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2"/>
       <c r="K21" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L21" s="2" t="s">
-        <v>177</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L21" s="2"/>
     </row>
     <row r="22" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>178</v>
+        <v>129</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>140</v>
+        <v>101</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>179</v>
+        <v>130</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>165</v>
+        <v>120</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>180</v>
+        <v>131</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>181</v>
+        <v>132</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>182</v>
+        <v>133</v>
       </c>
       <c r="H22" s="2"/>
-      <c r="I22" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="J22" s="2" t="s">
-        <v>183</v>
-      </c>
+      <c r="I22" s="2"/>
+      <c r="J22" s="2"/>
       <c r="K22" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L22" s="2" t="s">
-        <v>138</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L22" s="2"/>
     </row>
     <row r="23" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>184</v>
+        <v>134</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>140</v>
+        <v>101</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>185</v>
+        <v>135</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>186</v>
+        <v>136</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>187</v>
+        <v>137</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>188</v>
+        <v>138</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>189</v>
+        <v>139</v>
       </c>
       <c r="H23" s="2"/>
-      <c r="I23" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="J23" s="2" t="s">
-        <v>191</v>
-      </c>
+      <c r="I23" s="2"/>
+      <c r="J23" s="2"/>
       <c r="K23" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L23" s="2" t="s">
-        <v>192</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L23" s="2"/>
     </row>
     <row r="24" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>193</v>
+        <v>140</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>194</v>
+        <v>141</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>195</v>
+        <v>142</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>196</v>
+        <v>143</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>197</v>
+        <v>144</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>198</v>
+        <v>145</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>199</v>
+        <v>146</v>
       </c>
       <c r="H24" s="2"/>
-      <c r="I24" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="J24" s="2" t="s">
-        <v>201</v>
-      </c>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
       <c r="K24" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L24" s="2" t="s">
-        <v>202</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L24" s="2"/>
     </row>
     <row r="25" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>203</v>
+        <v>147</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>194</v>
+        <v>141</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>204</v>
+        <v>148</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>196</v>
+        <v>143</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>205</v>
+        <v>149</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>206</v>
+        <v>150</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>207</v>
+        <v>151</v>
       </c>
       <c r="H25" s="2"/>
-      <c r="I25" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="J25" s="2" t="s">
-        <v>209</v>
-      </c>
+      <c r="I25" s="2"/>
+      <c r="J25" s="2"/>
       <c r="K25" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L25" s="2" t="s">
-        <v>210</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L25" s="2"/>
     </row>
     <row r="26" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>211</v>
+        <v>152</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>212</v>
+        <v>153</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>213</v>
+        <v>154</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>214</v>
+        <v>155</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>215</v>
+        <v>156</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>216</v>
+        <v>157</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>217</v>
+        <v>158</v>
       </c>
       <c r="H26" s="2"/>
-      <c r="I26" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="J26" s="2" t="s">
-        <v>219</v>
-      </c>
+      <c r="I26" s="2"/>
+      <c r="J26" s="2"/>
       <c r="K26" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L26" s="2" t="s">
-        <v>220</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L26" s="2"/>
     </row>
     <row r="27" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>221</v>
+        <v>159</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>212</v>
+        <v>153</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>222</v>
+        <v>160</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>214</v>
+        <v>155</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>223</v>
+        <v>161</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>224</v>
+        <v>162</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>225</v>
+        <v>163</v>
       </c>
       <c r="H27" s="2"/>
-      <c r="I27" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="J27" s="2" t="s">
-        <v>227</v>
-      </c>
+      <c r="I27" s="2"/>
+      <c r="J27" s="2"/>
       <c r="K27" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L27" s="2" t="s">
-        <v>228</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L27" s="2"/>
     </row>
     <row r="28" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>229</v>
+        <v>164</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>212</v>
+        <v>153</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>230</v>
+        <v>165</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>214</v>
+        <v>155</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>231</v>
+        <v>166</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>232</v>
+        <v>167</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>233</v>
+        <v>168</v>
       </c>
       <c r="H28" s="2"/>
-      <c r="I28" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="J28" s="2" t="s">
-        <v>235</v>
-      </c>
+      <c r="I28" s="2"/>
+      <c r="J28" s="2"/>
       <c r="K28" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L28" s="2" t="s">
-        <v>236</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L28" s="2"/>
     </row>
     <row r="29" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>237</v>
+        <v>169</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>212</v>
+        <v>153</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>238</v>
+        <v>170</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>214</v>
+        <v>155</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>239</v>
+        <v>171</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>240</v>
+        <v>172</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>241</v>
+        <v>173</v>
       </c>
       <c r="H29" s="2"/>
-      <c r="I29" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="J29" s="2" t="s">
-        <v>243</v>
-      </c>
+      <c r="I29" s="2"/>
+      <c r="J29" s="2"/>
       <c r="K29" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L29" s="2" t="s">
-        <v>244</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L29" s="2"/>
     </row>
     <row r="30" ht="111.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>245</v>
+        <v>174</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>246</v>
+        <v>175</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>247</v>
+        <v>176</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>248</v>
+        <v>177</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>249</v>
+        <v>178</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>250</v>
+        <v>179</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>251</v>
+        <v>180</v>
       </c>
       <c r="H30" s="2"/>
-      <c r="I30" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="J30" s="2" t="s">
-        <v>252</v>
-      </c>
+      <c r="I30" s="2"/>
+      <c r="J30" s="2"/>
       <c r="K30" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="L30" s="2" t="s">
-        <v>49</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L30" s="2"/>
     </row>
     <row r="31" ht="111.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>253</v>
+        <v>181</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>246</v>
+        <v>175</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>254</v>
+        <v>182</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>255</v>
+        <v>183</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>256</v>
+        <v>184</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>257</v>
+        <v>185</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>258</v>
+        <v>186</v>
       </c>
       <c r="H31" s="2"/>
-      <c r="I31" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="J31" s="2" t="s">
-        <v>259</v>
-      </c>
+      <c r="I31" s="2"/>
+      <c r="J31" s="2"/>
       <c r="K31" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="L31" s="2" t="s">
-        <v>49</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L31" s="2"/>
     </row>
     <row r="32" ht="111.75" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>260</v>
+        <v>187</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>246</v>
+        <v>175</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>261</v>
+        <v>188</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>262</v>
+        <v>189</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>263</v>
+        <v>190</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>264</v>
+        <v>191</v>
       </c>
       <c r="H32" s="2"/>
-      <c r="I32" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="J32" s="2" t="s">
-        <v>266</v>
-      </c>
+      <c r="I32" s="2"/>
+      <c r="J32" s="2"/>
       <c r="K32" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L32" s="2" t="s">
-        <v>236</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L32" s="2"/>
     </row>
     <row r="33" ht="84" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>267</v>
+        <v>192</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>246</v>
+        <v>175</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>268</v>
+        <v>193</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>269</v>
+        <v>194</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>270</v>
+        <v>195</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>271</v>
+        <v>196</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>272</v>
+        <v>197</v>
       </c>
       <c r="H33" s="2"/>
-      <c r="I33" s="2" t="s">
-        <v>273</v>
-      </c>
-      <c r="J33" s="2" t="s">
-        <v>273</v>
-      </c>
+      <c r="I33" s="2"/>
+      <c r="J33" s="2"/>
       <c r="K33" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="L33" s="2" t="s">
-        <v>49</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L33" s="2"/>
     </row>
     <row r="34" ht="97.5" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>274</v>
+        <v>198</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>275</v>
+        <v>199</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>276</v>
+        <v>200</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>151</v>
+        <v>109</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>143</v>
+        <v>104</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>277</v>
+        <v>201</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>278</v>
+        <v>202</v>
       </c>
       <c r="H34" s="2"/>
-      <c r="I34" s="2" t="s">
-        <v>279</v>
-      </c>
-      <c r="J34" s="2" t="s">
-        <v>280</v>
-      </c>
+      <c r="I34" s="2"/>
+      <c r="J34" s="2"/>
       <c r="K34" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L34" s="2" t="s">
-        <v>281</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L34" s="2"/>
     </row>
     <row r="35" ht="97.5" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>282</v>
+        <v>203</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>275</v>
+        <v>199</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>283</v>
+        <v>204</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>284</v>
+        <v>205</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>285</v>
+        <v>206</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>286</v>
+        <v>207</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>287</v>
+        <v>208</v>
       </c>
       <c r="H35" s="2"/>
-      <c r="I35" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="J35" s="2" t="s">
-        <v>289</v>
-      </c>
+      <c r="I35" s="2"/>
+      <c r="J35" s="2"/>
       <c r="K35" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L35" s="2" t="s">
-        <v>290</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L35" s="2"/>
     </row>
     <row r="36" ht="97.5" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>291</v>
+        <v>209</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>275</v>
+        <v>199</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>292</v>
+        <v>210</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>293</v>
+        <v>211</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>294</v>
+        <v>212</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>295</v>
+        <v>213</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>296</v>
+        <v>214</v>
       </c>
       <c r="H36" s="2"/>
-      <c r="I36" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="J36" s="2" t="s">
-        <v>297</v>
-      </c>
+      <c r="I36" s="2"/>
+      <c r="J36" s="2"/>
       <c r="K36" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="L36" s="2" t="s">
-        <v>49</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L36" s="2"/>
     </row>
     <row r="37" ht="97.5" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>298</v>
+        <v>215</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>275</v>
+        <v>199</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>299</v>
+        <v>216</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>300</v>
+        <v>217</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>301</v>
+        <v>218</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>302</v>
+        <v>219</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>303</v>
+        <v>220</v>
       </c>
       <c r="H37" s="2"/>
-      <c r="I37" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="J37" s="2" t="s">
-        <v>304</v>
-      </c>
+      <c r="I37" s="2"/>
+      <c r="J37" s="2"/>
       <c r="K37" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="L37" s="2" t="s">
-        <v>49</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="L37" s="2"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L37"/>
@@ -2870,90 +2405,90 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>305</v>
+        <v>221</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>306</v>
+        <v>222</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>307</v>
+        <v>223</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>308</v>
+        <v>224</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>309</v>
+        <v>225</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>308</v>
+        <v>224</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>310</v>
+        <v>226</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>311</v>
+        <v>227</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>312</v>
+        <v>228</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>313</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>314</v>
+        <v>230</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>315</v>
+        <v>231</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>316</v>
+        <v>232</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>317</v>
+        <v>233</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>318</v>
+        <v>234</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>319</v>
+        <v>235</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>320</v>
+        <v>236</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>321</v>
+        <v>237</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>322</v>
+        <v>238</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>323</v>
+        <v>239</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>324</v>
+        <v>240</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>325</v>
+        <v>241</v>
       </c>
     </row>
   </sheetData>
@@ -2976,12 +2511,12 @@
         <v>10</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>326</v>
+        <v>242</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>48</v>
+        <v>243</v>
       </c>
       <c r="B2" s="5">
         <f>COUNTIF('News CSS Test Cases'!$K$2:$K$37,A2)</f>
@@ -2990,7 +2525,7 @@
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B3" s="5">
         <f>COUNTIF('News CSS Test Cases'!$K$2:$K$37,A3)</f>
@@ -2999,7 +2534,7 @@
     </row>
     <row r="4" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>327</v>
+        <v>244</v>
       </c>
       <c r="B4" s="5">
         <f>COUNTIF('News CSS Test Cases'!$K$2:$K$37,A4)</f>
@@ -3008,7 +2543,7 @@
     </row>
     <row r="5" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>328</v>
+        <v>245</v>
       </c>
       <c r="B5" s="5">
         <f>COUNTIF('News CSS Test Cases'!$K$2:$K$37,A5)</f>
@@ -3017,7 +2552,7 @@
     </row>
     <row r="6" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>329</v>
+        <v>246</v>
       </c>
       <c r="B6" s="6">
         <f>SUM(B2:B5)</f>

</xml_diff>